<commit_message>
Actualizacion Plantilla de costos
</commit_message>
<xml_diff>
--- a/Plantilla de costos.xlsx
+++ b/Plantilla de costos.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\3315783\Gear-Eagle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4005DD28-3B56-49BF-B0A7-59FCDFAF15DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD28E42F-5874-486E-90B6-A1648488812A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F6A12270-2864-41C2-9158-BB7C559B5FBD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F6A12270-2864-41C2-9158-BB7C559B5FBD}"/>
   </bookViews>
   <sheets>
-    <sheet name="Roles" sheetId="3" r:id="rId1"/>
-    <sheet name="Estimacion por tareas" sheetId="2" r:id="rId2"/>
-    <sheet name="Costos de fase" sheetId="4" r:id="rId3"/>
-    <sheet name="Cronograma" sheetId="5" r:id="rId4"/>
+    <sheet name="Personal" sheetId="3" r:id="rId1"/>
+    <sheet name="Equipos de computo" sheetId="6" r:id="rId2"/>
+    <sheet name="Servidores" sheetId="7" r:id="rId3"/>
+    <sheet name="Estimacion por tareas" sheetId="2" r:id="rId4"/>
+    <sheet name="Costos de fase" sheetId="4" r:id="rId5"/>
+    <sheet name="Cronograma" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="113">
   <si>
     <t>Concepto</t>
   </si>
@@ -254,6 +255,132 @@
   </si>
   <si>
     <t>SALARIO-HONORARIOS</t>
+  </si>
+  <si>
+    <t>Procesador</t>
+  </si>
+  <si>
+    <t>Memoria RAM</t>
+  </si>
+  <si>
+    <t>Almacenamiento</t>
+  </si>
+  <si>
+    <t>Windows 11 Pro</t>
+  </si>
+  <si>
+    <t>Gráficos</t>
+  </si>
+  <si>
+    <t>Pantalla</t>
+  </si>
+  <si>
+    <t>Conectividad</t>
+  </si>
+  <si>
+    <t>Sistema operativo</t>
+  </si>
+  <si>
+    <t>Puertos</t>
+  </si>
+  <si>
+    <t>Batería</t>
+  </si>
+  <si>
+    <t>Peso</t>
+  </si>
+  <si>
+    <t>FICHA TECNICA DE EQUIPO</t>
+  </si>
+  <si>
+    <t>}</t>
+  </si>
+  <si>
+    <t>Intel Core i5-13420H (8 núcleos, hasta 4.6 GHz)</t>
+  </si>
+  <si>
+    <t>Campo</t>
+  </si>
+  <si>
+    <t>Especificación</t>
+  </si>
+  <si>
+    <t>16 GB DDR4</t>
+  </si>
+  <si>
+    <t>1 TB SSD NVMe</t>
+  </si>
+  <si>
+    <t>Intel UHD Graphics</t>
+  </si>
+  <si>
+    <t>15.6” Full HD (1920x1080)</t>
+  </si>
+  <si>
+    <t>Windows 11 Home/Pro</t>
+  </si>
+  <si>
+    <t>WiFi 6, Bluetooth 5.1</t>
+  </si>
+  <si>
+    <t>USB-C, USB 3.2, HDMI, RJ-45</t>
+  </si>
+  <si>
+    <t>~38 Wh (6–8 horas)</t>
+  </si>
+  <si>
+    <t>~1.65 kg</t>
+  </si>
+  <si>
+    <t>Intel Core i7-1355U (10 núcleos)</t>
+  </si>
+  <si>
+    <t>16 GB DDR4 (expandible a 32 GB)</t>
+  </si>
+  <si>
+    <t>512 GB SSD NVMe</t>
+  </si>
+  <si>
+    <t>Intel Iris Xe</t>
+  </si>
+  <si>
+    <t>13.3” Full HD</t>
+  </si>
+  <si>
+    <t>WiFi 6E, Bluetooth 5.2</t>
+  </si>
+  <si>
+    <t>USB-C (Thunderbolt), USB-A, HDMI</t>
+  </si>
+  <si>
+    <t>~54 Wh (8–10 horas)</t>
+  </si>
+  <si>
+    <t>~1.3 kg</t>
+  </si>
+  <si>
+    <t>Intel Core i7-1360P (12 núcleos)</t>
+  </si>
+  <si>
+    <t>16 GB DDR5 (expandible a 64 GB)</t>
+  </si>
+  <si>
+    <t>512 GB SSD NVMe (expandible)</t>
+  </si>
+  <si>
+    <t>16” WUXGA (1920x1200)</t>
+  </si>
+  <si>
+    <t>WiFi 6E, Bluetooth 5.3</t>
+  </si>
+  <si>
+    <t>Thunderbolt 4, USB-C, USB-A, HDMI</t>
+  </si>
+  <si>
+    <t>~51 Wh (hasta 10 horas)</t>
+  </si>
+  <si>
+    <t>~1.7 kg</t>
   </si>
 </sst>
 </file>
@@ -650,7 +777,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -731,33 +858,6 @@
     <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -809,31 +909,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -848,20 +927,286 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="38">
+    <dxf>
+      <numFmt numFmtId="165" formatCode="_-[$$-240A]\ * #,##0_-;\-[$$-240A]\ * #,##0_-;_-[$$-240A]\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="_-[$$-240A]\ * #,##0_-;\-[$$-240A]\ * #,##0_-;_-[$$-240A]\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="_-[$$-240A]\ * #,##0_-;\-[$$-240A]\ * #,##0_-;_-[$$-240A]\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-[$$-240A]\ * #,##0.00_-;\-[$$-240A]\ * #,##0.00_-;_-[$$-240A]\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -948,24 +1293,24 @@
       </border>
     </dxf>
     <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <border>
         <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
           <color indexed="64"/>
         </bottom>
       </border>
@@ -1056,24 +1401,24 @@
       </border>
     </dxf>
     <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <border>
         <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
           <color indexed="64"/>
         </bottom>
       </border>
@@ -1164,24 +1509,24 @@
       </border>
     </dxf>
     <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <border>
         <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
           <color indexed="64"/>
         </bottom>
       </border>
@@ -1221,203 +1566,6 @@
         </horizontal>
       </border>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$$-240A]\ * #,##0.00_-;\-[$$-240A]\ * #,##0.00_-;_-[$$-240A]\ * &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="_-[$$-240A]\ * #,##0_-;\-[$$-240A]\ * #,##0_-;_-[$$-240A]\ * &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="_-[$$-240A]\ * #,##0_-;\-[$$-240A]\ * #,##0_-;_-[$$-240A]\ * &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="_-[$$-240A]\ * #,##0_-;\-[$$-240A]\ * #,##0_-;_-[$$-240A]\ * &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1432,59 +1580,59 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{5741B42D-CDC8-4108-90F6-1DE69A655878}" name="Tabla410" displayName="Tabla410" ref="B9:C15" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="22" tableBorderDxfId="23" totalsRowBorderDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{5741B42D-CDC8-4108-90F6-1DE69A655878}" name="Tabla410" displayName="Tabla410" ref="B9:C15" totalsRowShown="0" headerRowDxfId="37" headerRowBorderDxfId="36" tableBorderDxfId="35" totalsRowBorderDxfId="34">
   <autoFilter ref="B9:C15" xr:uid="{5741B42D-CDC8-4108-90F6-1DE69A655878}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{E92B9558-BA0E-4D64-8542-12DD024C8043}" name="Concepto" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{8851DFA3-212D-491C-91A7-C7C20F1707B8}" name="Valor" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{E92B9558-BA0E-4D64-8542-12DD024C8043}" name="Concepto" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{8851DFA3-212D-491C-91A7-C7C20F1707B8}" name="Valor" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{0A0E5314-895C-4C9A-9A33-0B2B25A668B4}" name="Tabla4611" displayName="Tabla4611" ref="B17:C23" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="4" tableBorderDxfId="5" totalsRowBorderDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{0A0E5314-895C-4C9A-9A33-0B2B25A668B4}" name="Tabla4611" displayName="Tabla4611" ref="B17:C23" totalsRowShown="0" headerRowDxfId="31" headerRowBorderDxfId="30" tableBorderDxfId="29" totalsRowBorderDxfId="28">
   <autoFilter ref="B17:C23" xr:uid="{0A0E5314-895C-4C9A-9A33-0B2B25A668B4}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{F2B70788-3621-49CF-95D5-6199C2D91744}" name="Concepto" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{D7BB54E9-3E44-4F87-B1BD-EB18A796F884}" name="Valor" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{F2B70788-3621-49CF-95D5-6199C2D91744}" name="Concepto" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{D7BB54E9-3E44-4F87-B1BD-EB18A796F884}" name="Valor" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{DD8576B5-BDC3-4437-ABB1-95052E3F828C}" name="Tabla4812" displayName="Tabla4812" ref="B25:C31" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="10" tableBorderDxfId="11" totalsRowBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{DD8576B5-BDC3-4437-ABB1-95052E3F828C}" name="Tabla4812" displayName="Tabla4812" ref="B25:C31" totalsRowShown="0" headerRowDxfId="25" headerRowBorderDxfId="24" tableBorderDxfId="23" totalsRowBorderDxfId="22">
   <autoFilter ref="B25:C31" xr:uid="{DD8576B5-BDC3-4437-ABB1-95052E3F828C}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{FD5C9B93-C029-4DC6-BC3A-A21E1D7681DA}" name="Concepto" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{9B141DC3-060F-4B05-93BB-A0C0D1ED8431}" name="Valor" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{FD5C9B93-C029-4DC6-BC3A-A21E1D7681DA}" name="Concepto" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{9B141DC3-060F-4B05-93BB-A0C0D1ED8431}" name="Valor" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{7ECDE91C-8104-4186-B165-D02FFF5FFE25}" name="Tabla4913" displayName="Tabla4913" ref="B33:C39" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="16" tableBorderDxfId="17" totalsRowBorderDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{7ECDE91C-8104-4186-B165-D02FFF5FFE25}" name="Tabla4913" displayName="Tabla4913" ref="B33:C39" totalsRowShown="0" headerRowDxfId="19" headerRowBorderDxfId="18" tableBorderDxfId="17" totalsRowBorderDxfId="16">
   <autoFilter ref="B33:C39" xr:uid="{7ECDE91C-8104-4186-B165-D02FFF5FFE25}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C457AEB7-D5AE-46CD-96C0-59F8C1177259}" name="Concepto" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{FFFBAA01-81EF-43AF-906B-1897360B8FE5}" name="Valor" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{C457AEB7-D5AE-46CD-96C0-59F8C1177259}" name="Concepto" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{FFFBAA01-81EF-43AF-906B-1897360B8FE5}" name="Valor" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C4F95F23-BE9F-4356-9A8D-6942ABC7C73A}" name="Tabla3" displayName="Tabla3" ref="B2:G10" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C4F95F23-BE9F-4356-9A8D-6942ABC7C73A}" name="Tabla3" displayName="Tabla3" ref="B2:G10" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="B2:G10" xr:uid="{C4F95F23-BE9F-4356-9A8D-6942ABC7C73A}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{71965BB9-5C68-4904-9229-4D3A1AC66DFC}" name="ID" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{084B4B35-4D55-49A6-AF4E-B09D63134F2B}" name="Tarea" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{A240D6BA-1B5C-41E3-BF2B-755DDFCB3C36}" name="Fase" dataDxfId="35"/>
-    <tableColumn id="4" xr3:uid="{ED811CF4-C430-47A6-960F-4B9A5D327148}" name="Horas estimadas" dataDxfId="28"/>
-    <tableColumn id="5" xr3:uid="{47C57152-A6EB-4249-B7B7-A76F939E0198}" name="Tarifa hora" dataDxfId="27" dataCellStyle="Millares"/>
-    <tableColumn id="6" xr3:uid="{D31B676D-D444-4E2E-8DDA-8880CF45F3F9}" name="Costo" dataDxfId="26" dataCellStyle="Millares">
+    <tableColumn id="1" xr3:uid="{71965BB9-5C68-4904-9229-4D3A1AC66DFC}" name="ID" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{084B4B35-4D55-49A6-AF4E-B09D63134F2B}" name="Tarea" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{A240D6BA-1B5C-41E3-BF2B-755DDFCB3C36}" name="Fase" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{ED811CF4-C430-47A6-960F-4B9A5D327148}" name="Horas estimadas" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{47C57152-A6EB-4249-B7B7-A76F939E0198}" name="Tarifa hora" dataDxfId="7" dataCellStyle="Millares"/>
+    <tableColumn id="6" xr3:uid="{D31B676D-D444-4E2E-8DDA-8880CF45F3F9}" name="Costo" dataDxfId="6" dataCellStyle="Millares">
       <calculatedColumnFormula>E3*F3</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1493,12 +1641,12 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A2AC0C33-2B67-4536-AD93-6AE14C6D86EA}" name="Tabla1" displayName="Tabla1" ref="B3:D8" totalsRowShown="0" headerRowBorderDxfId="34" tableBorderDxfId="33" totalsRowBorderDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A2AC0C33-2B67-4536-AD93-6AE14C6D86EA}" name="Tabla1" displayName="Tabla1" ref="B3:D8" totalsRowShown="0" headerRowBorderDxfId="5" tableBorderDxfId="4" totalsRowBorderDxfId="3">
   <autoFilter ref="B3:D8" xr:uid="{A2AC0C33-2B67-4536-AD93-6AE14C6D86EA}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{DCDFF22A-A6A9-4ACC-80B8-F31F18723EA6}" name="Fase" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{7B6F93FD-F67E-458F-8B98-F1EED99E1183}" name="Descripción" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{4DF75085-883B-4EE1-BD8F-AD7C4BFEC0B4}" name="Costo" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{DCDFF22A-A6A9-4ACC-80B8-F31F18723EA6}" name="Fase" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{7B6F93FD-F67E-458F-8B98-F1EED99E1183}" name="Descripción" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{4DF75085-883B-4EE1-BD8F-AD7C4BFEC0B4}" name="Costo" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1839,43 +1987,43 @@
   <sheetData>
     <row r="1" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="39" t="s">
+      <c r="C2" s="69" t="s">
         <v>70</v>
       </c>
-      <c r="D2" s="81" t="s">
+      <c r="D2" s="83" t="s">
         <v>68</v>
       </c>
-      <c r="E2" s="36" t="s">
+      <c r="E2" s="82" t="s">
         <v>48</v>
       </c>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36" t="s">
+      <c r="F2" s="82"/>
+      <c r="G2" s="82"/>
+      <c r="H2" s="82" t="s">
         <v>49</v>
       </c>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="64" t="s">
+      <c r="I2" s="82"/>
+      <c r="J2" s="82"/>
+      <c r="K2" s="82"/>
+      <c r="L2" s="75" t="s">
         <v>50</v>
       </c>
-      <c r="M2" s="65"/>
-      <c r="N2" s="66"/>
-      <c r="O2" s="34" t="s">
+      <c r="M2" s="76"/>
+      <c r="N2" s="77"/>
+      <c r="O2" s="78" t="s">
         <v>56</v>
       </c>
-      <c r="P2" s="41" t="s">
+      <c r="P2" s="80" t="s">
         <v>59</v>
       </c>
-      <c r="Q2" s="83"/>
+      <c r="Q2" s="65"/>
     </row>
     <row r="3" spans="2:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="38"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="82"/>
+      <c r="B3" s="68"/>
+      <c r="C3" s="70"/>
+      <c r="D3" s="84"/>
       <c r="E3" s="18" t="s">
         <v>52</v>
       </c>
@@ -1906,9 +2054,9 @@
       <c r="N3" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="O3" s="35"/>
-      <c r="P3" s="42"/>
-      <c r="Q3" s="83"/>
+      <c r="O3" s="79"/>
+      <c r="P3" s="81"/>
+      <c r="Q3" s="65"/>
     </row>
     <row r="4" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B4" s="19" t="s">
@@ -1998,7 +2146,7 @@
         <v>120000</v>
       </c>
       <c r="M5" s="26">
-        <f t="shared" ref="M5:M7" si="0">C5*0.03</f>
+        <f t="shared" ref="M5:M6" si="0">C5*0.03</f>
         <v>90000</v>
       </c>
       <c r="N5" s="26">
@@ -2040,7 +2188,7 @@
         <v>666400</v>
       </c>
       <c r="J6" s="26">
-        <f t="shared" ref="J6:J7" si="3">C6*0.01</f>
+        <f t="shared" ref="J6" si="3">C6*0.01</f>
         <v>80000</v>
       </c>
       <c r="K6" s="26">
@@ -2054,7 +2202,7 @@
         <v>240000</v>
       </c>
       <c r="N6" s="26">
-        <f t="shared" ref="N6:N7" si="4">C6*0.02</f>
+        <f t="shared" ref="N6" si="4">C6*0.02</f>
         <v>160000</v>
       </c>
       <c r="O6" s="26">
@@ -2073,7 +2221,7 @@
       <c r="C7" s="24">
         <v>2800000</v>
       </c>
-      <c r="D7" s="84" t="s">
+      <c r="D7" s="66" t="s">
         <v>67</v>
       </c>
       <c r="E7" s="28"/>
@@ -2096,35 +2244,35 @@
       </c>
     </row>
     <row r="9" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="51" t="s">
+      <c r="B9" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="52" t="s">
+      <c r="C9" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="D9" s="75"/>
+      <c r="D9" s="59"/>
     </row>
     <row r="10" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B10" s="53" t="s">
+      <c r="B10" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="54">
+      <c r="C10" s="45">
         <v>3200000</v>
       </c>
-      <c r="D10" s="76"/>
+      <c r="D10" s="60"/>
       <c r="F10" s="71" t="s">
         <v>62</v>
       </c>
       <c r="G10" s="72"/>
     </row>
     <row r="11" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B11" s="55" t="s">
+      <c r="B11" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="56">
+      <c r="C11" s="47">
         <v>160</v>
       </c>
-      <c r="D11" s="77"/>
+      <c r="D11" s="61"/>
       <c r="E11" s="5"/>
       <c r="F11" s="73"/>
       <c r="G11" s="74"/>
@@ -2137,28 +2285,28 @@
       <c r="N11" s="32"/>
     </row>
     <row r="12" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B12" s="55" t="s">
+      <c r="B12" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="57">
+      <c r="C12" s="48">
         <f>C10/160</f>
         <v>20000</v>
       </c>
-      <c r="D12" s="78"/>
-      <c r="F12" s="67" t="s">
+      <c r="D12" s="62"/>
+      <c r="F12" s="55" t="s">
         <v>60</v>
       </c>
-      <c r="G12" s="61" t="s">
+      <c r="G12" s="52" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="13" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B13" s="55" t="s">
+      <c r="B13" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="58"/>
-      <c r="D13" s="79"/>
-      <c r="F13" s="68" t="s">
+      <c r="C13" s="49"/>
+      <c r="D13" s="63"/>
+      <c r="F13" s="56" t="s">
         <v>26</v>
       </c>
       <c r="G13" s="27">
@@ -2167,26 +2315,26 @@
       </c>
     </row>
     <row r="14" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B14" s="55" t="s">
+      <c r="B14" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="56"/>
-      <c r="D14" s="77"/>
-      <c r="F14" s="69" t="s">
+      <c r="C14" s="47"/>
+      <c r="D14" s="61"/>
+      <c r="F14" s="57" t="s">
         <v>27</v>
       </c>
       <c r="G14" s="27">
-        <f t="shared" ref="G14:G16" si="5">O5*12</f>
+        <f t="shared" ref="G14:G15" si="5">O5*12</f>
         <v>54666720</v>
       </c>
     </row>
     <row r="15" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B15" s="59" t="s">
+      <c r="B15" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="60"/>
-      <c r="D15" s="79"/>
-      <c r="F15" s="68" t="s">
+      <c r="C15" s="51"/>
+      <c r="D15" s="63"/>
+      <c r="F15" s="56" t="s">
         <v>28</v>
       </c>
       <c r="G15" s="27">
@@ -2198,7 +2346,7 @@
       <c r="B16" s="6"/>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
-      <c r="F16" s="70" t="s">
+      <c r="F16" s="58" t="s">
         <v>29</v>
       </c>
       <c r="G16" s="29">
@@ -2206,201 +2354,204 @@
         <v>2800000</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="51" t="s">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C17" s="52" t="s">
+      <c r="C17" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="D17" s="75"/>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B18" s="55" t="s">
+      <c r="D17" s="59"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B18" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="C18" s="58">
+      <c r="C18" s="49">
         <v>3000000</v>
       </c>
-      <c r="D18" s="79"/>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B19" s="55" t="s">
+      <c r="D18" s="63"/>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B19" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="C19" s="56">
+      <c r="C19" s="47">
         <v>160</v>
       </c>
-      <c r="D19" s="77"/>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B20" s="55" t="s">
+      <c r="D19" s="61"/>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B20" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="C20" s="58">
+      <c r="C20" s="49">
         <f>C18/C19</f>
         <v>18750</v>
       </c>
-      <c r="D20" s="79"/>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B21" s="55" t="s">
+      <c r="D20" s="63"/>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B21" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="C21" s="58"/>
-      <c r="D21" s="79"/>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B22" s="55" t="s">
+      <c r="C21" s="49"/>
+      <c r="D21" s="63"/>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="C22" s="56"/>
-      <c r="D22" s="77"/>
-    </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B23" s="59" t="s">
+      <c r="C22" s="47"/>
+      <c r="D22" s="61"/>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B23" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="C23" s="60"/>
-      <c r="D23" s="79"/>
-    </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C23" s="51"/>
+      <c r="D23" s="63"/>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="6"/>
       <c r="C24" s="7"/>
       <c r="D24" s="7"/>
-    </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B25" s="51" t="s">
+      <c r="F24" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B25" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C25" s="52" t="s">
+      <c r="C25" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="D25" s="75"/>
-    </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B26" s="53" t="s">
+      <c r="D25" s="59"/>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B26" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="54">
+      <c r="C26" s="45">
         <v>8000000</v>
       </c>
-      <c r="D26" s="76"/>
-    </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B27" s="55" t="s">
+      <c r="D26" s="60"/>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B27" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="C27" s="56">
+      <c r="C27" s="47">
         <v>160</v>
       </c>
-      <c r="D27" s="77"/>
-    </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B28" s="55" t="s">
+      <c r="D27" s="61"/>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B28" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="C28" s="58">
+      <c r="C28" s="49">
         <f>C26/160</f>
         <v>50000</v>
       </c>
-      <c r="D28" s="79"/>
-    </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B29" s="55" t="s">
+      <c r="D28" s="63"/>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B29" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="C29" s="58"/>
-      <c r="D29" s="79"/>
-    </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B30" s="55" t="s">
+      <c r="C29" s="49"/>
+      <c r="D29" s="63"/>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B30" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="C30" s="56"/>
-      <c r="D30" s="77"/>
-    </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B31" s="59" t="s">
+      <c r="C30" s="47"/>
+      <c r="D30" s="61"/>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B31" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="C31" s="60"/>
-      <c r="D31" s="79"/>
-    </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C31" s="51"/>
+      <c r="D31" s="63"/>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B32" s="6"/>
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B33" s="51" t="s">
+      <c r="B33" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C33" s="52" t="s">
+      <c r="C33" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="D33" s="75"/>
+      <c r="D33" s="59"/>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B34" s="62" t="s">
+      <c r="B34" s="53" t="s">
         <v>29</v>
       </c>
-      <c r="C34" s="63">
+      <c r="C34" s="54">
         <v>2800000</v>
       </c>
-      <c r="D34" s="80"/>
+      <c r="D34" s="64"/>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B35" s="55" t="s">
+      <c r="B35" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="C35" s="56">
+      <c r="C35" s="47">
         <v>160</v>
       </c>
-      <c r="D35" s="77"/>
+      <c r="D35" s="61"/>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B36" s="55" t="s">
+      <c r="B36" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="C36" s="58">
+      <c r="C36" s="49">
         <f>C34/160</f>
         <v>17500</v>
       </c>
-      <c r="D36" s="79"/>
+      <c r="D36" s="63"/>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B37" s="55" t="s">
+      <c r="B37" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="C37" s="58"/>
-      <c r="D37" s="79"/>
+      <c r="C37" s="49"/>
+      <c r="D37" s="63"/>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B38" s="55" t="s">
+      <c r="B38" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="C38" s="56"/>
-      <c r="D38" s="77"/>
+      <c r="C38" s="47"/>
+      <c r="D38" s="61"/>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B39" s="59" t="s">
+      <c r="B39" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="C39" s="60"/>
-      <c r="D39" s="79"/>
+      <c r="C39" s="51"/>
+      <c r="D39" s="63"/>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:K2"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="F10:G11"/>
     <mergeCell ref="L2:N2"/>
     <mergeCell ref="O2:O3"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:K2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2414,6 +2565,306 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{611B09A3-7F71-49EA-AE70-97B3169F4335}">
+  <dimension ref="B2:F29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="23.140625" customWidth="1"/>
+    <col min="3" max="3" width="62.85546875" customWidth="1"/>
+    <col min="5" max="5" width="21.28515625" customWidth="1"/>
+    <col min="6" max="6" width="59.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="71" t="s">
+        <v>82</v>
+      </c>
+      <c r="C3" s="72"/>
+      <c r="E3" s="71" t="s">
+        <v>82</v>
+      </c>
+      <c r="F3" s="72"/>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="73"/>
+      <c r="C4" s="74"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="74"/>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="88" t="s">
+        <v>85</v>
+      </c>
+      <c r="C5" s="85" t="s">
+        <v>86</v>
+      </c>
+      <c r="E5" s="88" t="s">
+        <v>85</v>
+      </c>
+      <c r="F5" s="91" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="89" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" s="86" t="s">
+        <v>84</v>
+      </c>
+      <c r="E6" s="89" t="s">
+        <v>71</v>
+      </c>
+      <c r="F6" s="86" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="86" t="s">
+        <v>87</v>
+      </c>
+      <c r="E7" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="F7" s="86" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="89" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" s="86" t="s">
+        <v>88</v>
+      </c>
+      <c r="E8" s="89" t="s">
+        <v>73</v>
+      </c>
+      <c r="F8" s="86" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="89" t="s">
+        <v>75</v>
+      </c>
+      <c r="C9" s="86" t="s">
+        <v>89</v>
+      </c>
+      <c r="E9" s="89" t="s">
+        <v>75</v>
+      </c>
+      <c r="F9" s="86" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="89" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="86" t="s">
+        <v>90</v>
+      </c>
+      <c r="E10" s="89" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" s="86" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="89" t="s">
+        <v>78</v>
+      </c>
+      <c r="C11" s="86" t="s">
+        <v>91</v>
+      </c>
+      <c r="E11" s="89" t="s">
+        <v>78</v>
+      </c>
+      <c r="F11" s="86" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B12" s="89" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="86" t="s">
+        <v>92</v>
+      </c>
+      <c r="E12" s="89" t="s">
+        <v>77</v>
+      </c>
+      <c r="F12" s="86" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B13" s="89" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" s="86" t="s">
+        <v>93</v>
+      </c>
+      <c r="E13" s="89" t="s">
+        <v>79</v>
+      </c>
+      <c r="F13" s="86" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B14" s="89" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" s="86" t="s">
+        <v>94</v>
+      </c>
+      <c r="E14" s="89" t="s">
+        <v>80</v>
+      </c>
+      <c r="F14" s="86" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="90" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" s="87" t="s">
+        <v>95</v>
+      </c>
+      <c r="E15" s="90" t="s">
+        <v>81</v>
+      </c>
+      <c r="F15" s="87" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" s="71" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" s="72"/>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18" s="73"/>
+      <c r="C18" s="74"/>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="88" t="s">
+        <v>85</v>
+      </c>
+      <c r="C19" s="91" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B20" s="89" t="s">
+        <v>71</v>
+      </c>
+      <c r="C20" s="86" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B21" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" s="86" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B22" s="89" t="s">
+        <v>73</v>
+      </c>
+      <c r="C22" s="86" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B23" s="89" t="s">
+        <v>75</v>
+      </c>
+      <c r="C23" s="86" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B24" s="89" t="s">
+        <v>76</v>
+      </c>
+      <c r="C24" s="86" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B25" s="89" t="s">
+        <v>78</v>
+      </c>
+      <c r="C25" s="86" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B26" s="89" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="86" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B27" s="89" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" s="86" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B28" s="89" t="s">
+        <v>80</v>
+      </c>
+      <c r="C28" s="86" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="90" t="s">
+        <v>81</v>
+      </c>
+      <c r="C29" s="87" t="s">
+        <v>112</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B3:C4"/>
+    <mergeCell ref="E3:F4"/>
+    <mergeCell ref="B17:C18"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBB7ED60-6EC3-445B-A2DD-E27E6C31149E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6EAF1EC-B720-46EF-8B96-415750F7DB87}">
   <dimension ref="B2:G10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2422,8 +2873,8 @@
     <col min="3" max="3" width="25.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" style="50" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" style="50" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" style="41" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" style="41" customWidth="1"/>
     <col min="10" max="10" width="28.140625" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
     <col min="12" max="12" width="24" customWidth="1"/>
@@ -2444,10 +2895,10 @@
       <c r="E2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="48" t="s">
+      <c r="F2" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="48" t="s">
+      <c r="G2" s="39" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2464,10 +2915,10 @@
       <c r="E3" s="1">
         <v>6</v>
       </c>
-      <c r="F3" s="49">
+      <c r="F3" s="40">
         <v>25000</v>
       </c>
-      <c r="G3" s="49">
+      <c r="G3" s="40">
         <f t="shared" ref="G3:G10" si="0">E3*F3</f>
         <v>150000</v>
       </c>
@@ -2485,10 +2936,10 @@
       <c r="E4" s="1">
         <v>8</v>
       </c>
-      <c r="F4" s="49">
+      <c r="F4" s="40">
         <v>25000</v>
       </c>
-      <c r="G4" s="49">
+      <c r="G4" s="40">
         <f t="shared" si="0"/>
         <v>200000</v>
       </c>
@@ -2506,10 +2957,10 @@
       <c r="E5" s="1">
         <v>10</v>
       </c>
-      <c r="F5" s="49">
+      <c r="F5" s="40">
         <v>25000</v>
       </c>
-      <c r="G5" s="49">
+      <c r="G5" s="40">
         <f t="shared" si="0"/>
         <v>250000</v>
       </c>
@@ -2527,10 +2978,10 @@
       <c r="E6" s="1">
         <v>20</v>
       </c>
-      <c r="F6" s="49">
+      <c r="F6" s="40">
         <v>25000</v>
       </c>
-      <c r="G6" s="49">
+      <c r="G6" s="40">
         <f t="shared" si="0"/>
         <v>500000</v>
       </c>
@@ -2548,10 +2999,10 @@
       <c r="E7" s="1">
         <v>20</v>
       </c>
-      <c r="F7" s="49">
+      <c r="F7" s="40">
         <v>25000</v>
       </c>
-      <c r="G7" s="49">
+      <c r="G7" s="40">
         <f t="shared" si="0"/>
         <v>500000</v>
       </c>
@@ -2569,10 +3020,10 @@
       <c r="E8" s="1">
         <v>6</v>
       </c>
-      <c r="F8" s="49">
+      <c r="F8" s="40">
         <v>25000</v>
       </c>
-      <c r="G8" s="49">
+      <c r="G8" s="40">
         <f t="shared" si="0"/>
         <v>150000</v>
       </c>
@@ -2590,10 +3041,10 @@
       <c r="E9" s="1">
         <v>8</v>
       </c>
-      <c r="F9" s="49">
+      <c r="F9" s="40">
         <v>25000</v>
       </c>
-      <c r="G9" s="49">
+      <c r="G9" s="40">
         <f t="shared" si="0"/>
         <v>200000</v>
       </c>
@@ -2611,10 +3062,10 @@
       <c r="E10" s="1">
         <v>6</v>
       </c>
-      <c r="F10" s="49">
+      <c r="F10" s="40">
         <v>25000</v>
       </c>
-      <c r="G10" s="49">
+      <c r="G10" s="40">
         <f t="shared" si="0"/>
         <v>150000</v>
       </c>
@@ -2627,7 +3078,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B16C6EAF-BAFA-4751-A60D-13E5CA8A5F6C}">
   <dimension ref="B1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2635,17 +3086,17 @@
     <col min="1" max="1" width="11.42578125" style="6"/>
     <col min="2" max="2" width="19.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14" style="47" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14" style="38" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="11.42578125" style="6"/>
     <col min="7" max="9" width="11.42578125" style="6" customWidth="1"/>
     <col min="10" max="16384" width="11.42578125" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D1" s="43"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="2:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D2" s="43"/>
+      <c r="D2" s="34"/>
     </row>
     <row r="3" spans="2:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="14" t="s">
@@ -2654,7 +3105,7 @@
       <c r="C3" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="44" t="s">
+      <c r="D3" s="35" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2665,7 +3116,7 @@
       <c r="C4" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="D4" s="45">
+      <c r="D4" s="36">
         <v>150000</v>
       </c>
     </row>
@@ -2676,7 +3127,7 @@
       <c r="C5" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="45">
+      <c r="D5" s="36">
         <v>450000</v>
       </c>
     </row>
@@ -2687,7 +3138,7 @@
       <c r="C6" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="45">
+      <c r="D6" s="36">
         <v>1150000</v>
       </c>
     </row>
@@ -2698,7 +3149,7 @@
       <c r="C7" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="45">
+      <c r="D7" s="36">
         <v>200000</v>
       </c>
     </row>
@@ -2709,7 +3160,7 @@
       <c r="C8" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="46">
+      <c r="D8" s="37">
         <v>150000</v>
       </c>
     </row>
@@ -2724,7 +3175,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB354C72-A85A-4861-A24D-E3C392F56913}">
   <dimension ref="B3:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>